<commit_message>
New constraint rule: Subset of standard times
A course the rule names is not flagged for meeting on only some of the days of a standard time (same
start and length). Without the rule such a meeting is flagged, and the flag says when the rule would
allow it. The editor, the Constraints tab, the Excel format, the demo schedule and the docs know about it.

Assisted by Claude Sonnet 5.5 (Anthropic).
</commit_message>
<xml_diff>
--- a/apps/web/public/examples/example-schedule-revised.xlsx
+++ b/apps/web/public/examples/example-schedule-revised.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1301" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="236">
   <si>
     <t>Term</t>
   </si>
@@ -697,7 +697,7 @@
     <t>Export Time</t>
   </si>
   <si>
-    <t>10:29:00</t>
+    <t>22:57:57</t>
   </si>
   <si>
     <t>Academic Year</t>
@@ -716,6 +716,9 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>Default Department</t>
   </si>
   <si>
     <t>Version</t>
@@ -5616,7 +5619,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -5703,6 +5706,14 @@
         <v>19</v>
       </c>
     </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>235</v>
+      </c>
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Examples and the constraint-rules demo use made-up prefixes, numbers and titles
AMUS, BHAV, CRUD, DIGI and HELP replace MATH, STAT, CS, DATA and CORE,
course numbers are renumbered at the same level, and titles are invented.
The Help examples follow.

Assisted by Claude Sonnet 5.5 (Anthropic).
</commit_message>
<xml_diff>
--- a/apps/web/public/examples/example-schedule-revised.xlsx
+++ b/apps/web/public/examples/example-schedule-revised.xlsx
@@ -124,10 +124,10 @@
     <t>Advising coordinator</t>
   </si>
   <si>
-    <t>DATA</t>
-  </si>
-  <si>
-    <t>202</t>
+    <t>AMUS</t>
+  </si>
+  <si>
+    <t>112</t>
   </si>
   <si>
     <t>A</t>
@@ -136,261 +136,261 @@
     <t>4</t>
   </si>
   <si>
+    <t>MWF</t>
+  </si>
+  <si>
+    <t>09:15:00 - 10:20:00</t>
+  </si>
+  <si>
+    <t>NH 101</t>
+  </si>
+  <si>
+    <t>Musical Patterns I</t>
+  </si>
+  <si>
+    <t>Lecture</t>
+  </si>
+  <si>
+    <t>In-Person</t>
+  </si>
+  <si>
+    <t>SU</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>MTWRF</t>
+  </si>
+  <si>
+    <t>09:00:00 - 11:30:00</t>
+  </si>
+  <si>
+    <t>Second</t>
+  </si>
+  <si>
+    <t>SU-Second</t>
+  </si>
+  <si>
+    <t>Summer session II</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>12:15:00 - 13:20:00</t>
+  </si>
+  <si>
+    <t>119</t>
+  </si>
+  <si>
+    <t>Musical Patterns I (second semester)</t>
+  </si>
+  <si>
+    <t>145</t>
+  </si>
+  <si>
+    <t>NH 102</t>
+  </si>
+  <si>
+    <t>Musical Patterns II</t>
+  </si>
+  <si>
+    <t>WI</t>
+  </si>
+  <si>
+    <t>181</t>
+  </si>
+  <si>
+    <t>WI-Full</t>
+  </si>
+  <si>
+    <t>Algorithms and Music</t>
+  </si>
+  <si>
+    <t>Cy Fictional</t>
+  </si>
+  <si>
+    <t>Winter intensive: meets every weekday for two weeks</t>
+  </si>
+  <si>
+    <t>203</t>
+  </si>
+  <si>
+    <t>08:00:00 - 09:05:00</t>
+  </si>
+  <si>
+    <t>NH 103</t>
+  </si>
+  <si>
+    <t>Discrete Rhythm</t>
+  </si>
+  <si>
+    <t>228</t>
+  </si>
+  <si>
     <t>TR</t>
   </si>
   <si>
+    <t>10:20:00 - 12:00:00</t>
+  </si>
+  <si>
+    <t>Harmonic Structures</t>
+  </si>
+  <si>
+    <t>235</t>
+  </si>
+  <si>
+    <t>Multivoice Analysis</t>
+  </si>
+  <si>
+    <t>368</t>
+  </si>
+  <si>
+    <t>14:10:00 - 15:50:00</t>
+  </si>
+  <si>
+    <t>NH 104</t>
+  </si>
+  <si>
+    <t>Corpus Studies I</t>
+  </si>
+  <si>
+    <t>375</t>
+  </si>
+  <si>
+    <t>Corpus Studies II</t>
+  </si>
+  <si>
+    <t>BHAV</t>
+  </si>
+  <si>
+    <t>13:30:00 - 14:35:00</t>
+  </si>
+  <si>
+    <t>NH 105</t>
+  </si>
+  <si>
+    <t>Introduction to Behavioral Dynamics</t>
+  </si>
+  <si>
+    <t>Dee Placeholder</t>
+  </si>
+  <si>
+    <t>First</t>
+  </si>
+  <si>
+    <t>SU-First</t>
+  </si>
+  <si>
+    <t>Online</t>
+  </si>
+  <si>
+    <t>Summer session I</t>
+  </si>
+  <si>
+    <t>121</t>
+  </si>
+  <si>
+    <t>13:00:00 - 15:30:00</t>
+  </si>
+  <si>
+    <t>Behavior in Sport</t>
+  </si>
+  <si>
+    <t>212</t>
+  </si>
+  <si>
+    <t>Behavioral Methods</t>
+  </si>
+  <si>
+    <t>219</t>
+  </si>
+  <si>
+    <t>Models of Change</t>
+  </si>
+  <si>
+    <t>312</t>
+  </si>
+  <si>
+    <t>12:15:00 - 13:55:00</t>
+  </si>
+  <si>
+    <t>Stochastic Behavior</t>
+  </si>
+  <si>
+    <t>Eli Specimen, Dee Placeholder</t>
+  </si>
+  <si>
+    <t>DIGI</t>
+  </si>
+  <si>
+    <t>225</t>
+  </si>
+  <si>
     <t>08:00:00 - 09:40:00</t>
   </si>
   <si>
     <t>SB 110</t>
   </si>
   <si>
-    <t>Data Computing</t>
+    <t>Information Computing</t>
   </si>
   <si>
     <t>Fay Mockson</t>
   </si>
   <si>
-    <t>Lecture</t>
-  </si>
-  <si>
-    <t>In-Person</t>
-  </si>
-  <si>
-    <t>301</t>
-  </si>
-  <si>
-    <t>MWF</t>
+    <t>306</t>
   </si>
   <si>
     <t>11:00:00 - 12:05:00</t>
   </si>
   <si>
-    <t>Machine Learning</t>
-  </si>
-  <si>
-    <t>302</t>
-  </si>
-  <si>
-    <t>12:15:00 - 13:55:00</t>
-  </si>
-  <si>
-    <t>Data Science Capstone</t>
-  </si>
-  <si>
-    <t>380</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>14:10:00 - 15:50:00</t>
-  </si>
-  <si>
-    <t>First</t>
+    <t>Network Optimization</t>
+  </si>
+  <si>
+    <t>Also listed as BHAV 306</t>
+  </si>
+  <si>
+    <t>BHAV 306</t>
+  </si>
+  <si>
+    <t>318</t>
+  </si>
+  <si>
+    <t>Adaptive Systems</t>
+  </si>
+  <si>
+    <t>325</t>
+  </si>
+  <si>
+    <t>Information Capstone</t>
+  </si>
+  <si>
+    <t>371</t>
   </si>
   <si>
     <t>FA-First</t>
   </si>
   <si>
-    <t>Data Ethics</t>
+    <t>Information Ethics</t>
   </si>
   <si>
     <t>First half of the term</t>
   </si>
   <si>
-    <t>381</t>
-  </si>
-  <si>
-    <t>Second</t>
+    <t>378</t>
   </si>
   <si>
     <t>FA-Second</t>
   </si>
   <si>
-    <t>Data Visualization</t>
+    <t>Information Visualization</t>
   </si>
   <si>
     <t>Second half of the term</t>
   </si>
   <si>
-    <t>385</t>
-  </si>
-  <si>
-    <t>Optimization</t>
-  </si>
-  <si>
-    <t>Also listed as STAT 385</t>
-  </si>
-  <si>
-    <t>STAT 385</t>
-  </si>
-  <si>
-    <t>WI</t>
-  </si>
-  <si>
-    <t>MATH</t>
-  </si>
-  <si>
-    <t>110</t>
-  </si>
-  <si>
-    <t>MTWRF</t>
-  </si>
-  <si>
-    <t>09:00:00 - 11:30:00</t>
-  </si>
-  <si>
-    <t>NH 101</t>
-  </si>
-  <si>
-    <t>WI-Full</t>
-  </si>
-  <si>
-    <t>Mathematics and Music</t>
-  </si>
-  <si>
-    <t>Cy Fictional</t>
-  </si>
-  <si>
-    <t>Winter intensive: meets every weekday for two weeks</t>
-  </si>
-  <si>
-    <t>143</t>
-  </si>
-  <si>
-    <t>09:15:00 - 10:20:00</t>
-  </si>
-  <si>
-    <t>Calculus I</t>
-  </si>
-  <si>
-    <t>SU</t>
-  </si>
-  <si>
-    <t>SU-Second</t>
-  </si>
-  <si>
-    <t>Summer session II</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>12:15:00 - 13:20:00</t>
-  </si>
-  <si>
-    <t>144</t>
-  </si>
-  <si>
-    <t>Calculus I (second semester)</t>
-  </si>
-  <si>
-    <t>162</t>
-  </si>
-  <si>
-    <t>NH 102</t>
-  </si>
-  <si>
-    <t>Calculus II</t>
-  </si>
-  <si>
-    <t>231</t>
-  </si>
-  <si>
-    <t>10:20:00 - 12:00:00</t>
-  </si>
-  <si>
-    <t>NH 103</t>
-  </si>
-  <si>
-    <t>Linear Algebra</t>
-  </si>
-  <si>
-    <t>232</t>
-  </si>
-  <si>
-    <t>Multivariable Calculus</t>
-  </si>
-  <si>
-    <t>256</t>
-  </si>
-  <si>
-    <t>08:00:00 - 09:05:00</t>
-  </si>
-  <si>
-    <t>Discrete Mathematics</t>
-  </si>
-  <si>
-    <t>351</t>
-  </si>
-  <si>
-    <t>NH 104</t>
-  </si>
-  <si>
-    <t>Real Analysis I</t>
-  </si>
-  <si>
-    <t>352</t>
-  </si>
-  <si>
-    <t>Real Analysis II</t>
-  </si>
-  <si>
-    <t>STAT</t>
-  </si>
-  <si>
-    <t>130</t>
-  </si>
-  <si>
-    <t>13:00:00 - 15:30:00</t>
-  </si>
-  <si>
-    <t>NH 105</t>
-  </si>
-  <si>
-    <t>Sports Analytics</t>
-  </si>
-  <si>
-    <t>13:30:00 - 14:35:00</t>
-  </si>
-  <si>
-    <t>Introduction to Statistics</t>
-  </si>
-  <si>
-    <t>Dee Placeholder</t>
-  </si>
-  <si>
-    <t>SU-First</t>
-  </si>
-  <si>
-    <t>Online</t>
-  </si>
-  <si>
-    <t>Summer session I</t>
-  </si>
-  <si>
-    <t>243</t>
-  </si>
-  <si>
-    <t>Statistical Methods</t>
-  </si>
-  <si>
-    <t>244</t>
-  </si>
-  <si>
-    <t>Regression</t>
-  </si>
-  <si>
-    <t>343</t>
-  </si>
-  <si>
-    <t>Probability</t>
-  </si>
-  <si>
-    <t>Eli Specimen, Dee Placeholder</t>
-  </si>
-  <si>
     <t>SectionId</t>
   </si>
   <si>
@@ -427,7 +427,7 @@
     <t>EnrollmentDay10</t>
   </si>
   <si>
-    <t>AY25-FA-MATH143-A</t>
+    <t>AY25-FA-AMUS112-A</t>
   </si>
   <si>
     <t>AY25</t>
@@ -436,100 +436,100 @@
     <t>09:15</t>
   </si>
   <si>
-    <t>AY25-FA-MATH143-B</t>
+    <t>AY25-FA-AMUS112-B</t>
   </si>
   <si>
     <t>12:15</t>
   </si>
   <si>
-    <t>AY25-FA-MATH162-A</t>
-  </si>
-  <si>
-    <t>AY25-FA-MATH231-A</t>
+    <t>AY25-FA-AMUS145-A</t>
+  </si>
+  <si>
+    <t>AY25-FA-AMUS228-A</t>
   </si>
   <si>
     <t>10:20</t>
   </si>
   <si>
-    <t>AY25-FA-MATH256-A</t>
+    <t>AY25-FA-AMUS203-A</t>
   </si>
   <si>
     <t>08:00</t>
   </si>
   <si>
-    <t>AY25-FA-MATH351-A</t>
+    <t>AY25-FA-AMUS368-A</t>
   </si>
   <si>
     <t>14:10</t>
   </si>
   <si>
-    <t>AY25-FA-STAT143-A</t>
+    <t>AY25-FA-BHAV112-A</t>
   </si>
   <si>
     <t>13:30</t>
   </si>
   <si>
-    <t>AY25-FA-STAT243-A</t>
-  </si>
-  <si>
-    <t>AY25-FA-STAT343-A</t>
-  </si>
-  <si>
-    <t>AY25-FA-DATA202-A</t>
-  </si>
-  <si>
-    <t>AY25-FA-DATA380-A</t>
-  </si>
-  <si>
-    <t>AY25-FA-DATA381-A</t>
-  </si>
-  <si>
-    <t>AY25-FA-DATA385-A</t>
+    <t>AY25-FA-BHAV212-A</t>
+  </si>
+  <si>
+    <t>AY25-FA-BHAV312-A</t>
+  </si>
+  <si>
+    <t>AY25-FA-DIGI225-A</t>
+  </si>
+  <si>
+    <t>AY25-FA-DIGI371-A</t>
+  </si>
+  <si>
+    <t>AY25-FA-DIGI378-A</t>
+  </si>
+  <si>
+    <t>AY25-FA-DIGI306-A</t>
   </si>
   <si>
     <t>11:00</t>
   </si>
   <si>
-    <t>AY25-WI-MATH110-A</t>
+    <t>AY25-WI-AMUS181-A</t>
   </si>
   <si>
     <t>09:00</t>
   </si>
   <si>
-    <t>AY25-WI-STAT130-A</t>
+    <t>AY25-WI-BHAV121-A</t>
   </si>
   <si>
     <t>13:00</t>
   </si>
   <si>
-    <t>AY25-SP-MATH144-A</t>
-  </si>
-  <si>
-    <t>AY25-SP-MATH162-A</t>
-  </si>
-  <si>
-    <t>AY25-SP-MATH232-A</t>
-  </si>
-  <si>
-    <t>AY25-SP-MATH352-A</t>
-  </si>
-  <si>
-    <t>AY25-SP-STAT143-A</t>
-  </si>
-  <si>
-    <t>AY25-SP-STAT244-A</t>
-  </si>
-  <si>
-    <t>AY25-SP-DATA301-A</t>
-  </si>
-  <si>
-    <t>AY25-SP-DATA302-A</t>
-  </si>
-  <si>
-    <t>AY25-SU-MATH143-A</t>
-  </si>
-  <si>
-    <t>AY25-SU-STAT143-A</t>
+    <t>AY25-SP-AMUS119-A</t>
+  </si>
+  <si>
+    <t>AY25-SP-AMUS145-A</t>
+  </si>
+  <si>
+    <t>AY25-SP-AMUS235-A</t>
+  </si>
+  <si>
+    <t>AY25-SP-AMUS375-A</t>
+  </si>
+  <si>
+    <t>AY25-SP-BHAV112-A</t>
+  </si>
+  <si>
+    <t>AY25-SP-BHAV219-A</t>
+  </si>
+  <si>
+    <t>AY25-SP-DIGI318-A</t>
+  </si>
+  <si>
+    <t>AY25-SP-DIGI325-A</t>
+  </si>
+  <si>
+    <t>AY25-SU-AMUS112-A</t>
+  </si>
+  <si>
+    <t>AY25-SU-BHAV112-A</t>
   </si>
   <si>
     <t>Activity</t>
@@ -691,13 +691,13 @@
     <t>Export Date</t>
   </si>
   <si>
-    <t>2026-10-03</t>
+    <t>2026-10-04</t>
   </si>
   <si>
     <t>Export Time</t>
   </si>
   <si>
-    <t>22:57:57</t>
+    <t>08:26:04</t>
   </si>
   <si>
     <t>Academic Year</t>
@@ -1118,7 +1118,7 @@
     <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="11" width="13" customWidth="1"/>
     <col min="12" max="12" width="10" customWidth="1"/>
-    <col min="13" max="13" width="30" customWidth="1"/>
+    <col min="13" max="13" width="38" customWidth="1"/>
     <col min="14" max="14" width="31" customWidth="1"/>
     <col min="15" max="15" width="22" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
@@ -1497,19 +1497,19 @@
         <v>23</v>
       </c>
       <c r="L7">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="M7" t="s">
         <v>42</v>
       </c>
       <c r="N7" t="s">
+        <v>24</v>
+      </c>
+      <c r="O7" t="s">
         <v>43</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>44</v>
-      </c>
-      <c r="P7" t="s">
-        <v>45</v>
       </c>
       <c r="Q7" t="s">
         <v>19</v>
@@ -1520,22 +1520,22 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
         <v>35</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
         <v>37</v>
       </c>
       <c r="E8" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="F8" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G8" t="s">
         <v>47</v>
@@ -1547,28 +1547,28 @@
         <v>41</v>
       </c>
       <c r="J8" t="s">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="K8" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="L8">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="M8" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="N8" t="s">
+        <v>30</v>
+      </c>
+      <c r="O8" t="s">
         <v>43</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>44</v>
       </c>
-      <c r="P8" t="s">
-        <v>45</v>
-      </c>
       <c r="Q8" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="R8" t="s">
         <v>19</v>
@@ -1576,16 +1576,16 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
         <v>35</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="E9" t="s">
         <v>38</v>
@@ -1597,7 +1597,7 @@
         <v>39</v>
       </c>
       <c r="H9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I9" t="s">
         <v>41</v>
@@ -1606,22 +1606,22 @@
         <v>22</v>
       </c>
       <c r="K9" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="L9">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="M9" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="N9" t="s">
+        <v>24</v>
+      </c>
+      <c r="O9" t="s">
         <v>43</v>
       </c>
-      <c r="O9" t="s">
+      <c r="P9" t="s">
         <v>44</v>
-      </c>
-      <c r="P9" t="s">
-        <v>45</v>
       </c>
       <c r="Q9" t="s">
         <v>19</v>
@@ -1632,55 +1632,55 @@
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
         <v>35</v>
       </c>
       <c r="C10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D10" t="s">
         <v>37</v>
       </c>
       <c r="E10" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="F10" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="G10" t="s">
         <v>39</v>
       </c>
       <c r="H10" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="I10" t="s">
         <v>41</v>
       </c>
       <c r="J10" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="K10" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="L10">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="M10" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="N10" t="s">
+        <v>24</v>
+      </c>
+      <c r="O10" t="s">
         <v>43</v>
       </c>
-      <c r="O10" t="s">
+      <c r="P10" t="s">
         <v>44</v>
       </c>
-      <c r="P10" t="s">
-        <v>45</v>
-      </c>
       <c r="Q10" t="s">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="R10" t="s">
         <v>19</v>
@@ -1694,49 +1694,49 @@
         <v>35</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D11" t="s">
         <v>37</v>
       </c>
       <c r="E11" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="F11" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="G11" t="s">
         <v>39</v>
       </c>
       <c r="H11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="I11" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="J11" t="s">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="K11" t="s">
-        <v>62</v>
+        <v>23</v>
       </c>
       <c r="L11">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="M11" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="N11" t="s">
+        <v>30</v>
+      </c>
+      <c r="O11" t="s">
         <v>43</v>
       </c>
-      <c r="O11" t="s">
+      <c r="P11" t="s">
         <v>44</v>
       </c>
-      <c r="P11" t="s">
-        <v>45</v>
-      </c>
       <c r="Q11" t="s">
-        <v>64</v>
+        <v>19</v>
       </c>
       <c r="R11" t="s">
         <v>19</v>
@@ -1744,13 +1744,13 @@
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
         <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="D12" t="s">
         <v>37</v>
@@ -1762,51 +1762,51 @@
         <v>38</v>
       </c>
       <c r="G12" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="H12" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="I12" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="J12" t="s">
         <v>22</v>
       </c>
       <c r="K12" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="L12">
         <v>65</v>
       </c>
       <c r="M12" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="N12" t="s">
+        <v>30</v>
+      </c>
+      <c r="O12" t="s">
         <v>43</v>
       </c>
-      <c r="O12" t="s">
+      <c r="P12" t="s">
         <v>44</v>
       </c>
-      <c r="P12" t="s">
-        <v>45</v>
-      </c>
       <c r="Q12" t="s">
-        <v>67</v>
+        <v>19</v>
       </c>
       <c r="R12" t="s">
-        <v>68</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="B13" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="D13" t="s">
         <v>37</v>
@@ -1818,37 +1818,37 @@
         <v>38</v>
       </c>
       <c r="G13" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="H13" t="s">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="I13" t="s">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="J13" t="s">
         <v>22</v>
       </c>
       <c r="K13" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="L13">
         <v>150</v>
       </c>
       <c r="M13" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="N13" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="O13" t="s">
+        <v>43</v>
+      </c>
+      <c r="P13" t="s">
         <v>44</v>
       </c>
-      <c r="P13" t="s">
-        <v>45</v>
-      </c>
       <c r="Q13" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="R13" t="s">
         <v>19</v>
@@ -1859,10 +1859,10 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="C14" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="D14" t="s">
         <v>37</v>
@@ -1874,13 +1874,13 @@
         <v>38</v>
       </c>
       <c r="G14" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="H14" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="I14" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="J14" t="s">
         <v>22</v>
@@ -1892,16 +1892,16 @@
         <v>65</v>
       </c>
       <c r="M14" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="N14" t="s">
-        <v>24</v>
+        <v>63</v>
       </c>
       <c r="O14" t="s">
+        <v>43</v>
+      </c>
+      <c r="P14" t="s">
         <v>44</v>
-      </c>
-      <c r="P14" t="s">
-        <v>45</v>
       </c>
       <c r="Q14" t="s">
         <v>19</v>
@@ -1912,55 +1912,55 @@
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>82</v>
+        <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="C15" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="D15" t="s">
         <v>37</v>
       </c>
       <c r="E15" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="F15" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="G15" t="s">
+        <v>70</v>
+      </c>
+      <c r="H15" t="s">
+        <v>71</v>
+      </c>
+      <c r="I15" t="s">
+        <v>67</v>
+      </c>
+      <c r="J15" t="s">
+        <v>22</v>
+      </c>
+      <c r="K15" t="s">
+        <v>23</v>
+      </c>
+      <c r="L15">
+        <v>100</v>
+      </c>
+      <c r="M15" t="s">
         <v>72</v>
       </c>
-      <c r="H15" t="s">
-        <v>73</v>
-      </c>
-      <c r="I15" t="s">
-        <v>74</v>
-      </c>
-      <c r="J15" t="s">
-        <v>61</v>
-      </c>
-      <c r="K15" t="s">
-        <v>83</v>
-      </c>
-      <c r="L15">
-        <v>150</v>
-      </c>
-      <c r="M15" t="s">
-        <v>81</v>
-      </c>
       <c r="N15" t="s">
-        <v>30</v>
+        <v>63</v>
       </c>
       <c r="O15" t="s">
+        <v>43</v>
+      </c>
+      <c r="P15" t="s">
         <v>44</v>
       </c>
-      <c r="P15" t="s">
-        <v>45</v>
-      </c>
       <c r="Q15" t="s">
-        <v>84</v>
+        <v>19</v>
       </c>
       <c r="R15" t="s">
         <v>19</v>
@@ -1968,16 +1968,16 @@
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="C16" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="D16" t="s">
-        <v>85</v>
+        <v>37</v>
       </c>
       <c r="E16" t="s">
         <v>38</v>
@@ -1986,34 +1986,34 @@
         <v>38</v>
       </c>
       <c r="G16" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="H16" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="I16" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="J16" t="s">
         <v>22</v>
       </c>
       <c r="K16" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="L16">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="M16" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="N16" t="s">
-        <v>24</v>
+        <v>63</v>
       </c>
       <c r="O16" t="s">
+        <v>43</v>
+      </c>
+      <c r="P16" t="s">
         <v>44</v>
-      </c>
-      <c r="P16" t="s">
-        <v>45</v>
       </c>
       <c r="Q16" t="s">
         <v>19</v>
@@ -2024,13 +2024,13 @@
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="C17" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="D17" t="s">
         <v>37</v>
@@ -2042,34 +2042,34 @@
         <v>38</v>
       </c>
       <c r="G17" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="H17" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I17" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="J17" t="s">
         <v>22</v>
       </c>
       <c r="K17" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="L17">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="M17" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="N17" t="s">
-        <v>24</v>
+        <v>63</v>
       </c>
       <c r="O17" t="s">
+        <v>43</v>
+      </c>
+      <c r="P17" t="s">
         <v>44</v>
-      </c>
-      <c r="P17" t="s">
-        <v>45</v>
       </c>
       <c r="Q17" t="s">
         <v>19</v>
@@ -2080,13 +2080,13 @@
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="C18" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="D18" t="s">
         <v>37</v>
@@ -2098,34 +2098,34 @@
         <v>38</v>
       </c>
       <c r="G18" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="H18" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="I18" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="J18" t="s">
         <v>22</v>
       </c>
       <c r="K18" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="L18">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="M18" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="N18" t="s">
         <v>30</v>
       </c>
       <c r="O18" t="s">
+        <v>43</v>
+      </c>
+      <c r="P18" t="s">
         <v>44</v>
-      </c>
-      <c r="P18" t="s">
-        <v>45</v>
       </c>
       <c r="Q18" t="s">
         <v>19</v>
@@ -2136,13 +2136,13 @@
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="C19" t="s">
-        <v>89</v>
+        <v>36</v>
       </c>
       <c r="D19" t="s">
         <v>37</v>
@@ -2154,34 +2154,34 @@
         <v>38</v>
       </c>
       <c r="G19" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="H19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I19" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="J19" t="s">
         <v>22</v>
       </c>
       <c r="K19" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="L19">
         <v>65</v>
       </c>
       <c r="M19" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="N19" t="s">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="O19" t="s">
+        <v>43</v>
+      </c>
+      <c r="P19" t="s">
         <v>44</v>
-      </c>
-      <c r="P19" t="s">
-        <v>45</v>
       </c>
       <c r="Q19" t="s">
         <v>19</v>
@@ -2192,13 +2192,13 @@
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="C20" t="s">
-        <v>92</v>
+        <v>36</v>
       </c>
       <c r="D20" t="s">
         <v>37</v>
@@ -2213,31 +2213,31 @@
         <v>39</v>
       </c>
       <c r="H20" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="I20" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="J20" t="s">
         <v>22</v>
       </c>
       <c r="K20" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="L20">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="M20" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="N20" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="O20" t="s">
+        <v>43</v>
+      </c>
+      <c r="P20" t="s">
         <v>44</v>
-      </c>
-      <c r="P20" t="s">
-        <v>45</v>
       </c>
       <c r="Q20" t="s">
         <v>19</v>
@@ -2248,55 +2248,55 @@
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="C21" t="s">
-        <v>96</v>
+        <v>36</v>
       </c>
       <c r="D21" t="s">
         <v>37</v>
       </c>
       <c r="E21" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="F21" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G21" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="H21" t="s">
-        <v>93</v>
+        <v>48</v>
       </c>
       <c r="I21" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="J21" t="s">
-        <v>22</v>
+        <v>86</v>
       </c>
       <c r="K21" t="s">
-        <v>28</v>
+        <v>87</v>
       </c>
       <c r="L21">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="M21" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="N21" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="O21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="P21" t="s">
-        <v>45</v>
+        <v>88</v>
       </c>
       <c r="Q21" t="s">
-        <v>19</v>
+        <v>89</v>
       </c>
       <c r="R21" t="s">
         <v>19</v>
@@ -2304,13 +2304,13 @@
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="B22" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="C22" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D22" t="s">
         <v>37</v>
@@ -2325,31 +2325,31 @@
         <v>47</v>
       </c>
       <c r="H22" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="I22" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="J22" t="s">
         <v>22</v>
       </c>
       <c r="K22" t="s">
-        <v>23</v>
+        <v>61</v>
       </c>
       <c r="L22">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="M22" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="N22" t="s">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="O22" t="s">
+        <v>43</v>
+      </c>
+      <c r="P22" t="s">
         <v>44</v>
-      </c>
-      <c r="P22" t="s">
-        <v>45</v>
       </c>
       <c r="Q22" t="s">
         <v>19</v>
@@ -2363,10 +2363,10 @@
         <v>18</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="C23" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="D23" t="s">
         <v>37</v>
@@ -2378,13 +2378,13 @@
         <v>38</v>
       </c>
       <c r="G23" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="H23" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="I23" t="s">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="J23" t="s">
         <v>22</v>
@@ -2396,16 +2396,16 @@
         <v>100</v>
       </c>
       <c r="M23" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="N23" t="s">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="O23" t="s">
+        <v>43</v>
+      </c>
+      <c r="P23" t="s">
         <v>44</v>
-      </c>
-      <c r="P23" t="s">
-        <v>45</v>
       </c>
       <c r="Q23" t="s">
         <v>19</v>
@@ -2419,10 +2419,10 @@
         <v>27</v>
       </c>
       <c r="B24" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="C24" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="D24" t="s">
         <v>37</v>
@@ -2434,13 +2434,13 @@
         <v>38</v>
       </c>
       <c r="G24" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="H24" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="I24" t="s">
-        <v>102</v>
+        <v>83</v>
       </c>
       <c r="J24" t="s">
         <v>22</v>
@@ -2452,16 +2452,16 @@
         <v>100</v>
       </c>
       <c r="M24" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="N24" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="O24" t="s">
+        <v>43</v>
+      </c>
+      <c r="P24" t="s">
         <v>44</v>
-      </c>
-      <c r="P24" t="s">
-        <v>45</v>
       </c>
       <c r="Q24" t="s">
         <v>19</v>
@@ -2472,13 +2472,13 @@
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="C25" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="D25" t="s">
         <v>37</v>
@@ -2490,34 +2490,34 @@
         <v>38</v>
       </c>
       <c r="G25" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H25" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I25" t="s">
-        <v>109</v>
+        <v>83</v>
       </c>
       <c r="J25" t="s">
         <v>22</v>
       </c>
       <c r="K25" t="s">
-        <v>75</v>
+        <v>23</v>
       </c>
       <c r="L25">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="M25" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="N25" t="s">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="O25" t="s">
+        <v>43</v>
+      </c>
+      <c r="P25" t="s">
         <v>44</v>
-      </c>
-      <c r="P25" t="s">
-        <v>45</v>
       </c>
       <c r="Q25" t="s">
         <v>19</v>
@@ -2531,10 +2531,10 @@
         <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C26" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="D26" t="s">
         <v>37</v>
@@ -2546,13 +2546,13 @@
         <v>38</v>
       </c>
       <c r="G26" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="H26" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="I26" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="J26" t="s">
         <v>22</v>
@@ -2561,19 +2561,19 @@
         <v>23</v>
       </c>
       <c r="L26">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="M26" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="N26" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="O26" t="s">
+        <v>43</v>
+      </c>
+      <c r="P26" t="s">
         <v>44</v>
-      </c>
-      <c r="P26" t="s">
-        <v>45</v>
       </c>
       <c r="Q26" t="s">
         <v>19</v>
@@ -2584,13 +2584,13 @@
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B27" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C27" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="D27" t="s">
         <v>37</v>
@@ -2602,93 +2602,93 @@
         <v>38</v>
       </c>
       <c r="G27" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="H27" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I27" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="J27" t="s">
         <v>22</v>
       </c>
       <c r="K27" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="L27">
         <v>65</v>
       </c>
       <c r="M27" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="N27" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="O27" t="s">
+        <v>43</v>
+      </c>
+      <c r="P27" t="s">
         <v>44</v>
       </c>
-      <c r="P27" t="s">
-        <v>45</v>
-      </c>
       <c r="Q27" t="s">
-        <v>19</v>
+        <v>110</v>
       </c>
       <c r="R27" t="s">
-        <v>19</v>
+        <v>111</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>82</v>
+        <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C28" t="s">
-        <v>79</v>
+        <v>112</v>
       </c>
       <c r="D28" t="s">
         <v>37</v>
       </c>
       <c r="E28" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="F28" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="G28" t="s">
-        <v>72</v>
+        <v>39</v>
       </c>
       <c r="H28" t="s">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="I28" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="J28" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="K28" t="s">
-        <v>114</v>
+        <v>28</v>
       </c>
       <c r="L28">
-        <v>150</v>
+        <v>65</v>
       </c>
       <c r="M28" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="N28" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="O28" t="s">
+        <v>43</v>
+      </c>
+      <c r="P28" t="s">
         <v>44</v>
       </c>
-      <c r="P28" t="s">
-        <v>115</v>
-      </c>
       <c r="Q28" t="s">
-        <v>116</v>
+        <v>19</v>
       </c>
       <c r="R28" t="s">
         <v>19</v>
@@ -2696,13 +2696,13 @@
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C29" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D29" t="s">
         <v>37</v>
@@ -2714,34 +2714,34 @@
         <v>38</v>
       </c>
       <c r="G29" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="H29" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="I29" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="J29" t="s">
         <v>22</v>
       </c>
       <c r="K29" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="L29">
         <v>100</v>
       </c>
       <c r="M29" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="N29" t="s">
-        <v>33</v>
+        <v>106</v>
       </c>
       <c r="O29" t="s">
+        <v>43</v>
+      </c>
+      <c r="P29" t="s">
         <v>44</v>
-      </c>
-      <c r="P29" t="s">
-        <v>45</v>
       </c>
       <c r="Q29" t="s">
         <v>19</v>
@@ -2752,55 +2752,55 @@
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B30" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C30" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D30" t="s">
         <v>37</v>
       </c>
       <c r="E30" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="F30" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G30" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="H30" t="s">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="I30" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="J30" t="s">
-        <v>22</v>
+        <v>86</v>
       </c>
       <c r="K30" t="s">
-        <v>28</v>
+        <v>117</v>
       </c>
       <c r="L30">
         <v>100</v>
       </c>
       <c r="M30" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="N30" t="s">
-        <v>33</v>
+        <v>106</v>
       </c>
       <c r="O30" t="s">
+        <v>43</v>
+      </c>
+      <c r="P30" t="s">
         <v>44</v>
       </c>
-      <c r="P30" t="s">
-        <v>45</v>
-      </c>
       <c r="Q30" t="s">
-        <v>19</v>
+        <v>119</v>
       </c>
       <c r="R30" t="s">
         <v>19</v>
@@ -2811,34 +2811,34 @@
         <v>18</v>
       </c>
       <c r="B31" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C31" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D31" t="s">
         <v>37</v>
       </c>
       <c r="E31" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="F31" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G31" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="H31" t="s">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="I31" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="J31" t="s">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="K31" t="s">
-        <v>23</v>
+        <v>121</v>
       </c>
       <c r="L31">
         <v>100</v>
@@ -2847,16 +2847,16 @@
         <v>122</v>
       </c>
       <c r="N31" t="s">
+        <v>106</v>
+      </c>
+      <c r="O31" t="s">
+        <v>43</v>
+      </c>
+      <c r="P31" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q31" t="s">
         <v>123</v>
-      </c>
-      <c r="O31" t="s">
-        <v>44</v>
-      </c>
-      <c r="P31" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q31" t="s">
-        <v>19</v>
       </c>
       <c r="R31" t="s">
         <v>19</v>
@@ -2887,7 +2887,7 @@
     <col min="14" max="14" width="11" customWidth="1"/>
     <col min="15" max="15" width="17" customWidth="1"/>
     <col min="16" max="16" width="11" customWidth="1"/>
-    <col min="17" max="17" width="30" customWidth="1"/>
+    <col min="17" max="17" width="38" customWidth="1"/>
     <col min="18" max="18" width="21" customWidth="1"/>
     <col min="19" max="19" width="13" customWidth="1"/>
     <col min="20" max="20" width="7" customWidth="1"/>
@@ -2988,10 +2988,10 @@
         <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="G2" t="s">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="H2" t="s">
         <v>37</v>
@@ -3009,7 +3009,7 @@
         <v>19</v>
       </c>
       <c r="M2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="N2" t="s">
         <v>138</v>
@@ -3018,22 +3018,22 @@
         <v>65</v>
       </c>
       <c r="P2" t="s">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="Q2" t="s">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="R2" t="s">
+        <v>43</v>
+      </c>
+      <c r="S2" t="s">
+        <v>19</v>
+      </c>
+      <c r="T2" t="s">
+        <v>19</v>
+      </c>
+      <c r="U2" t="s">
         <v>44</v>
-      </c>
-      <c r="S2" t="s">
-        <v>19</v>
-      </c>
-      <c r="T2" t="s">
-        <v>19</v>
-      </c>
-      <c r="U2" t="s">
-        <v>45</v>
       </c>
       <c r="V2" t="s">
         <v>19</v>
@@ -3062,13 +3062,13 @@
         <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="G3" t="s">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="H3" t="s">
-        <v>85</v>
+        <v>52</v>
       </c>
       <c r="I3" t="s">
         <v>24</v>
@@ -3083,7 +3083,7 @@
         <v>19</v>
       </c>
       <c r="M3" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="N3" t="s">
         <v>140</v>
@@ -3092,22 +3092,22 @@
         <v>65</v>
       </c>
       <c r="P3" t="s">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="Q3" t="s">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="R3" t="s">
+        <v>43</v>
+      </c>
+      <c r="S3" t="s">
+        <v>19</v>
+      </c>
+      <c r="T3" t="s">
+        <v>19</v>
+      </c>
+      <c r="U3" t="s">
         <v>44</v>
-      </c>
-      <c r="S3" t="s">
-        <v>19</v>
-      </c>
-      <c r="T3" t="s">
-        <v>19</v>
-      </c>
-      <c r="U3" t="s">
-        <v>45</v>
       </c>
       <c r="V3" t="s">
         <v>19</v>
@@ -3136,10 +3136,10 @@
         <v>22</v>
       </c>
       <c r="F4" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="G4" t="s">
-        <v>89</v>
+        <v>56</v>
       </c>
       <c r="H4" t="s">
         <v>37</v>
@@ -3157,7 +3157,7 @@
         <v>19</v>
       </c>
       <c r="M4" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="N4" t="s">
         <v>140</v>
@@ -3166,22 +3166,22 @@
         <v>65</v>
       </c>
       <c r="P4" t="s">
-        <v>90</v>
+        <v>57</v>
       </c>
       <c r="Q4" t="s">
-        <v>91</v>
+        <v>58</v>
       </c>
       <c r="R4" t="s">
+        <v>43</v>
+      </c>
+      <c r="S4" t="s">
+        <v>19</v>
+      </c>
+      <c r="T4" t="s">
+        <v>19</v>
+      </c>
+      <c r="U4" t="s">
         <v>44</v>
-      </c>
-      <c r="S4" t="s">
-        <v>19</v>
-      </c>
-      <c r="T4" t="s">
-        <v>19</v>
-      </c>
-      <c r="U4" t="s">
-        <v>45</v>
       </c>
       <c r="V4" t="s">
         <v>19</v>
@@ -3210,16 +3210,16 @@
         <v>22</v>
       </c>
       <c r="F5" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="G5" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="H5" t="s">
         <v>37</v>
       </c>
       <c r="I5" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -3231,7 +3231,7 @@
         <v>19</v>
       </c>
       <c r="M5" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="N5" t="s">
         <v>143</v>
@@ -3240,22 +3240,22 @@
         <v>100</v>
       </c>
       <c r="P5" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="Q5" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="R5" t="s">
+        <v>43</v>
+      </c>
+      <c r="S5" t="s">
+        <v>19</v>
+      </c>
+      <c r="T5" t="s">
+        <v>19</v>
+      </c>
+      <c r="U5" t="s">
         <v>44</v>
-      </c>
-      <c r="S5" t="s">
-        <v>19</v>
-      </c>
-      <c r="T5" t="s">
-        <v>19</v>
-      </c>
-      <c r="U5" t="s">
-        <v>45</v>
       </c>
       <c r="V5" t="s">
         <v>19</v>
@@ -3284,16 +3284,16 @@
         <v>22</v>
       </c>
       <c r="F6" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="G6" t="s">
-        <v>98</v>
+        <v>65</v>
       </c>
       <c r="H6" t="s">
         <v>37</v>
       </c>
       <c r="I6" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="J6">
         <v>4</v>
@@ -3305,7 +3305,7 @@
         <v>19</v>
       </c>
       <c r="M6" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="N6" t="s">
         <v>145</v>
@@ -3314,22 +3314,22 @@
         <v>65</v>
       </c>
       <c r="P6" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="Q6" t="s">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="R6" t="s">
+        <v>43</v>
+      </c>
+      <c r="S6" t="s">
+        <v>19</v>
+      </c>
+      <c r="T6" t="s">
+        <v>19</v>
+      </c>
+      <c r="U6" t="s">
         <v>44</v>
-      </c>
-      <c r="S6" t="s">
-        <v>19</v>
-      </c>
-      <c r="T6" t="s">
-        <v>19</v>
-      </c>
-      <c r="U6" t="s">
-        <v>45</v>
       </c>
       <c r="V6" t="s">
         <v>19</v>
@@ -3358,16 +3358,16 @@
         <v>22</v>
       </c>
       <c r="F7" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="G7" t="s">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="H7" t="s">
         <v>37</v>
       </c>
       <c r="I7" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="J7">
         <v>4</v>
@@ -3379,7 +3379,7 @@
         <v>19</v>
       </c>
       <c r="M7" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="N7" t="s">
         <v>147</v>
@@ -3388,22 +3388,22 @@
         <v>100</v>
       </c>
       <c r="P7" t="s">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="Q7" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="R7" t="s">
+        <v>43</v>
+      </c>
+      <c r="S7" t="s">
+        <v>19</v>
+      </c>
+      <c r="T7" t="s">
+        <v>19</v>
+      </c>
+      <c r="U7" t="s">
         <v>44</v>
-      </c>
-      <c r="S7" t="s">
-        <v>19</v>
-      </c>
-      <c r="T7" t="s">
-        <v>19</v>
-      </c>
-      <c r="U7" t="s">
-        <v>45</v>
       </c>
       <c r="V7" t="s">
         <v>19</v>
@@ -3432,16 +3432,16 @@
         <v>22</v>
       </c>
       <c r="F8" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="G8" t="s">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="H8" t="s">
         <v>37</v>
       </c>
       <c r="I8" t="s">
-        <v>113</v>
+        <v>85</v>
       </c>
       <c r="J8">
         <v>4</v>
@@ -3453,7 +3453,7 @@
         <v>19</v>
       </c>
       <c r="M8" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="N8" t="s">
         <v>149</v>
@@ -3462,22 +3462,22 @@
         <v>65</v>
       </c>
       <c r="P8" t="s">
-        <v>109</v>
+        <v>83</v>
       </c>
       <c r="Q8" t="s">
-        <v>112</v>
+        <v>84</v>
       </c>
       <c r="R8" t="s">
+        <v>43</v>
+      </c>
+      <c r="S8" t="s">
+        <v>19</v>
+      </c>
+      <c r="T8" t="s">
+        <v>19</v>
+      </c>
+      <c r="U8" t="s">
         <v>44</v>
-      </c>
-      <c r="S8" t="s">
-        <v>19</v>
-      </c>
-      <c r="T8" t="s">
-        <v>19</v>
-      </c>
-      <c r="U8" t="s">
-        <v>45</v>
       </c>
       <c r="V8" t="s">
         <v>19</v>
@@ -3506,10 +3506,10 @@
         <v>22</v>
       </c>
       <c r="F9" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="G9" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="H9" t="s">
         <v>37</v>
@@ -3527,7 +3527,7 @@
         <v>19</v>
       </c>
       <c r="M9" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="N9" t="s">
         <v>143</v>
@@ -3536,22 +3536,22 @@
         <v>100</v>
       </c>
       <c r="P9" t="s">
-        <v>109</v>
+        <v>83</v>
       </c>
       <c r="Q9" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="R9" t="s">
+        <v>43</v>
+      </c>
+      <c r="S9" t="s">
+        <v>19</v>
+      </c>
+      <c r="T9" t="s">
+        <v>19</v>
+      </c>
+      <c r="U9" t="s">
         <v>44</v>
-      </c>
-      <c r="S9" t="s">
-        <v>19</v>
-      </c>
-      <c r="T9" t="s">
-        <v>19</v>
-      </c>
-      <c r="U9" t="s">
-        <v>45</v>
       </c>
       <c r="V9" t="s">
         <v>19</v>
@@ -3580,16 +3580,16 @@
         <v>22</v>
       </c>
       <c r="F10" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="G10" t="s">
-        <v>121</v>
+        <v>97</v>
       </c>
       <c r="H10" t="s">
         <v>37</v>
       </c>
       <c r="I10" t="s">
-        <v>123</v>
+        <v>100</v>
       </c>
       <c r="J10">
         <v>4</v>
@@ -3601,7 +3601,7 @@
         <v>19</v>
       </c>
       <c r="M10" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="N10" t="s">
         <v>140</v>
@@ -3610,22 +3610,22 @@
         <v>100</v>
       </c>
       <c r="P10" t="s">
-        <v>109</v>
+        <v>83</v>
       </c>
       <c r="Q10" t="s">
-        <v>122</v>
+        <v>99</v>
       </c>
       <c r="R10" t="s">
+        <v>43</v>
+      </c>
+      <c r="S10" t="s">
+        <v>19</v>
+      </c>
+      <c r="T10" t="s">
+        <v>19</v>
+      </c>
+      <c r="U10" t="s">
         <v>44</v>
-      </c>
-      <c r="S10" t="s">
-        <v>19</v>
-      </c>
-      <c r="T10" t="s">
-        <v>19</v>
-      </c>
-      <c r="U10" t="s">
-        <v>45</v>
       </c>
       <c r="V10" t="s">
         <v>19</v>
@@ -3654,16 +3654,16 @@
         <v>22</v>
       </c>
       <c r="F11" t="s">
-        <v>35</v>
+        <v>101</v>
       </c>
       <c r="G11" t="s">
-        <v>36</v>
+        <v>102</v>
       </c>
       <c r="H11" t="s">
         <v>37</v>
       </c>
       <c r="I11" t="s">
-        <v>43</v>
+        <v>106</v>
       </c>
       <c r="J11">
         <v>4</v>
@@ -3675,7 +3675,7 @@
         <v>19</v>
       </c>
       <c r="M11" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="N11" t="s">
         <v>145</v>
@@ -3684,22 +3684,22 @@
         <v>100</v>
       </c>
       <c r="P11" t="s">
-        <v>41</v>
+        <v>104</v>
       </c>
       <c r="Q11" t="s">
-        <v>42</v>
+        <v>105</v>
       </c>
       <c r="R11" t="s">
+        <v>43</v>
+      </c>
+      <c r="S11" t="s">
+        <v>19</v>
+      </c>
+      <c r="T11" t="s">
+        <v>19</v>
+      </c>
+      <c r="U11" t="s">
         <v>44</v>
-      </c>
-      <c r="S11" t="s">
-        <v>19</v>
-      </c>
-      <c r="T11" t="s">
-        <v>19</v>
-      </c>
-      <c r="U11" t="s">
-        <v>45</v>
       </c>
       <c r="V11" t="s">
         <v>19</v>
@@ -3725,19 +3725,19 @@
         <v>18</v>
       </c>
       <c r="E12" t="s">
-        <v>56</v>
+        <v>86</v>
       </c>
       <c r="F12" t="s">
-        <v>35</v>
+        <v>101</v>
       </c>
       <c r="G12" t="s">
-        <v>53</v>
+        <v>116</v>
       </c>
       <c r="H12" t="s">
         <v>37</v>
       </c>
       <c r="I12" t="s">
-        <v>43</v>
+        <v>106</v>
       </c>
       <c r="J12">
         <v>2</v>
@@ -3749,7 +3749,7 @@
         <v>19</v>
       </c>
       <c r="M12" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="N12" t="s">
         <v>147</v>
@@ -3758,25 +3758,25 @@
         <v>100</v>
       </c>
       <c r="P12" t="s">
-        <v>41</v>
+        <v>104</v>
       </c>
       <c r="Q12" t="s">
-        <v>58</v>
+        <v>118</v>
       </c>
       <c r="R12" t="s">
+        <v>43</v>
+      </c>
+      <c r="S12" t="s">
+        <v>19</v>
+      </c>
+      <c r="T12" t="s">
+        <v>19</v>
+      </c>
+      <c r="U12" t="s">
         <v>44</v>
       </c>
-      <c r="S12" t="s">
-        <v>19</v>
-      </c>
-      <c r="T12" t="s">
-        <v>19</v>
-      </c>
-      <c r="U12" t="s">
-        <v>45</v>
-      </c>
       <c r="V12" t="s">
-        <v>59</v>
+        <v>119</v>
       </c>
       <c r="W12" t="s">
         <v>19</v>
@@ -3799,19 +3799,19 @@
         <v>18</v>
       </c>
       <c r="E13" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="F13" t="s">
-        <v>35</v>
+        <v>101</v>
       </c>
       <c r="G13" t="s">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="H13" t="s">
         <v>37</v>
       </c>
       <c r="I13" t="s">
-        <v>43</v>
+        <v>106</v>
       </c>
       <c r="J13">
         <v>2</v>
@@ -3823,7 +3823,7 @@
         <v>19</v>
       </c>
       <c r="M13" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="N13" t="s">
         <v>147</v>
@@ -3832,25 +3832,25 @@
         <v>100</v>
       </c>
       <c r="P13" t="s">
-        <v>41</v>
+        <v>104</v>
       </c>
       <c r="Q13" t="s">
-        <v>63</v>
+        <v>122</v>
       </c>
       <c r="R13" t="s">
+        <v>43</v>
+      </c>
+      <c r="S13" t="s">
+        <v>19</v>
+      </c>
+      <c r="T13" t="s">
+        <v>19</v>
+      </c>
+      <c r="U13" t="s">
         <v>44</v>
       </c>
-      <c r="S13" t="s">
-        <v>19</v>
-      </c>
-      <c r="T13" t="s">
-        <v>19</v>
-      </c>
-      <c r="U13" t="s">
-        <v>45</v>
-      </c>
       <c r="V13" t="s">
-        <v>64</v>
+        <v>123</v>
       </c>
       <c r="W13" t="s">
         <v>19</v>
@@ -3876,16 +3876,16 @@
         <v>22</v>
       </c>
       <c r="F14" t="s">
-        <v>35</v>
+        <v>101</v>
       </c>
       <c r="G14" t="s">
-        <v>65</v>
+        <v>107</v>
       </c>
       <c r="H14" t="s">
         <v>37</v>
       </c>
       <c r="I14" t="s">
-        <v>43</v>
+        <v>106</v>
       </c>
       <c r="J14">
         <v>4</v>
@@ -3897,7 +3897,7 @@
         <v>19</v>
       </c>
       <c r="M14" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="N14" t="s">
         <v>156</v>
@@ -3906,25 +3906,25 @@
         <v>65</v>
       </c>
       <c r="P14" t="s">
-        <v>41</v>
+        <v>104</v>
       </c>
       <c r="Q14" t="s">
-        <v>66</v>
+        <v>109</v>
       </c>
       <c r="R14" t="s">
+        <v>43</v>
+      </c>
+      <c r="S14" t="s">
+        <v>19</v>
+      </c>
+      <c r="T14" t="s">
+        <v>19</v>
+      </c>
+      <c r="U14" t="s">
         <v>44</v>
       </c>
-      <c r="S14" t="s">
-        <v>19</v>
-      </c>
-      <c r="T14" t="s">
-        <v>19</v>
-      </c>
-      <c r="U14" t="s">
-        <v>45</v>
-      </c>
       <c r="V14" t="s">
-        <v>67</v>
+        <v>110</v>
       </c>
       <c r="W14" t="s">
         <v>19</v>
@@ -3944,22 +3944,22 @@
         <v>137</v>
       </c>
       <c r="D15" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E15" t="s">
         <v>22</v>
       </c>
       <c r="F15" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="G15" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="H15" t="s">
         <v>37</v>
       </c>
       <c r="I15" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="J15">
         <v>4</v>
@@ -3971,7 +3971,7 @@
         <v>19</v>
       </c>
       <c r="M15" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="N15" t="s">
         <v>158</v>
@@ -3980,25 +3980,25 @@
         <v>150</v>
       </c>
       <c r="P15" t="s">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="Q15" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="R15" t="s">
+        <v>43</v>
+      </c>
+      <c r="S15" t="s">
+        <v>19</v>
+      </c>
+      <c r="T15" t="s">
+        <v>19</v>
+      </c>
+      <c r="U15" t="s">
         <v>44</v>
       </c>
-      <c r="S15" t="s">
-        <v>19</v>
-      </c>
-      <c r="T15" t="s">
-        <v>19</v>
-      </c>
-      <c r="U15" t="s">
-        <v>45</v>
-      </c>
       <c r="V15" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="W15" t="s">
         <v>19</v>
@@ -4018,16 +4018,16 @@
         <v>137</v>
       </c>
       <c r="D16" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E16" t="s">
         <v>22</v>
       </c>
       <c r="F16" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="G16" t="s">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="H16" t="s">
         <v>37</v>
@@ -4045,7 +4045,7 @@
         <v>19</v>
       </c>
       <c r="M16" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="N16" t="s">
         <v>160</v>
@@ -4054,22 +4054,22 @@
         <v>150</v>
       </c>
       <c r="P16" t="s">
-        <v>109</v>
+        <v>83</v>
       </c>
       <c r="Q16" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="R16" t="s">
+        <v>43</v>
+      </c>
+      <c r="S16" t="s">
+        <v>19</v>
+      </c>
+      <c r="T16" t="s">
+        <v>19</v>
+      </c>
+      <c r="U16" t="s">
         <v>44</v>
-      </c>
-      <c r="S16" t="s">
-        <v>19</v>
-      </c>
-      <c r="T16" t="s">
-        <v>19</v>
-      </c>
-      <c r="U16" t="s">
-        <v>45</v>
       </c>
       <c r="V16" t="s">
         <v>19</v>
@@ -4098,10 +4098,10 @@
         <v>22</v>
       </c>
       <c r="F17" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="G17" t="s">
-        <v>87</v>
+        <v>54</v>
       </c>
       <c r="H17" t="s">
         <v>37</v>
@@ -4119,7 +4119,7 @@
         <v>19</v>
       </c>
       <c r="M17" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="N17" t="s">
         <v>138</v>
@@ -4128,22 +4128,22 @@
         <v>65</v>
       </c>
       <c r="P17" t="s">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="Q17" t="s">
-        <v>88</v>
+        <v>55</v>
       </c>
       <c r="R17" t="s">
+        <v>43</v>
+      </c>
+      <c r="S17" t="s">
+        <v>19</v>
+      </c>
+      <c r="T17" t="s">
+        <v>19</v>
+      </c>
+      <c r="U17" t="s">
         <v>44</v>
-      </c>
-      <c r="S17" t="s">
-        <v>19</v>
-      </c>
-      <c r="T17" t="s">
-        <v>19</v>
-      </c>
-      <c r="U17" t="s">
-        <v>45</v>
       </c>
       <c r="V17" t="s">
         <v>19</v>
@@ -4172,10 +4172,10 @@
         <v>22</v>
       </c>
       <c r="F18" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="G18" t="s">
-        <v>89</v>
+        <v>56</v>
       </c>
       <c r="H18" t="s">
         <v>37</v>
@@ -4193,7 +4193,7 @@
         <v>19</v>
       </c>
       <c r="M18" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="N18" t="s">
         <v>138</v>
@@ -4202,22 +4202,22 @@
         <v>65</v>
       </c>
       <c r="P18" t="s">
-        <v>90</v>
+        <v>57</v>
       </c>
       <c r="Q18" t="s">
-        <v>91</v>
+        <v>58</v>
       </c>
       <c r="R18" t="s">
+        <v>43</v>
+      </c>
+      <c r="S18" t="s">
+        <v>19</v>
+      </c>
+      <c r="T18" t="s">
+        <v>19</v>
+      </c>
+      <c r="U18" t="s">
         <v>44</v>
-      </c>
-      <c r="S18" t="s">
-        <v>19</v>
-      </c>
-      <c r="T18" t="s">
-        <v>19</v>
-      </c>
-      <c r="U18" t="s">
-        <v>45</v>
       </c>
       <c r="V18" t="s">
         <v>19</v>
@@ -4246,16 +4246,16 @@
         <v>22</v>
       </c>
       <c r="F19" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="G19" t="s">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="H19" t="s">
         <v>37</v>
       </c>
       <c r="I19" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="J19">
         <v>4</v>
@@ -4267,7 +4267,7 @@
         <v>19</v>
       </c>
       <c r="M19" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="N19" t="s">
         <v>143</v>
@@ -4276,22 +4276,22 @@
         <v>100</v>
       </c>
       <c r="P19" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="Q19" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="R19" t="s">
+        <v>43</v>
+      </c>
+      <c r="S19" t="s">
+        <v>19</v>
+      </c>
+      <c r="T19" t="s">
+        <v>19</v>
+      </c>
+      <c r="U19" t="s">
         <v>44</v>
-      </c>
-      <c r="S19" t="s">
-        <v>19</v>
-      </c>
-      <c r="T19" t="s">
-        <v>19</v>
-      </c>
-      <c r="U19" t="s">
-        <v>45</v>
       </c>
       <c r="V19" t="s">
         <v>19</v>
@@ -4320,10 +4320,10 @@
         <v>22</v>
       </c>
       <c r="F20" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="G20" t="s">
-        <v>104</v>
+        <v>79</v>
       </c>
       <c r="H20" t="s">
         <v>37</v>
@@ -4341,7 +4341,7 @@
         <v>19</v>
       </c>
       <c r="M20" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="N20" t="s">
         <v>147</v>
@@ -4350,22 +4350,22 @@
         <v>100</v>
       </c>
       <c r="P20" t="s">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="Q20" t="s">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="R20" t="s">
+        <v>43</v>
+      </c>
+      <c r="S20" t="s">
+        <v>19</v>
+      </c>
+      <c r="T20" t="s">
+        <v>19</v>
+      </c>
+      <c r="U20" t="s">
         <v>44</v>
-      </c>
-      <c r="S20" t="s">
-        <v>19</v>
-      </c>
-      <c r="T20" t="s">
-        <v>19</v>
-      </c>
-      <c r="U20" t="s">
-        <v>45</v>
       </c>
       <c r="V20" t="s">
         <v>19</v>
@@ -4394,16 +4394,16 @@
         <v>22</v>
       </c>
       <c r="F21" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="G21" t="s">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="H21" t="s">
         <v>37</v>
       </c>
       <c r="I21" t="s">
-        <v>113</v>
+        <v>85</v>
       </c>
       <c r="J21">
         <v>4</v>
@@ -4415,7 +4415,7 @@
         <v>19</v>
       </c>
       <c r="M21" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="N21" t="s">
         <v>149</v>
@@ -4424,22 +4424,22 @@
         <v>65</v>
       </c>
       <c r="P21" t="s">
-        <v>109</v>
+        <v>83</v>
       </c>
       <c r="Q21" t="s">
-        <v>112</v>
+        <v>84</v>
       </c>
       <c r="R21" t="s">
+        <v>43</v>
+      </c>
+      <c r="S21" t="s">
+        <v>19</v>
+      </c>
+      <c r="T21" t="s">
+        <v>19</v>
+      </c>
+      <c r="U21" t="s">
         <v>44</v>
-      </c>
-      <c r="S21" t="s">
-        <v>19</v>
-      </c>
-      <c r="T21" t="s">
-        <v>19</v>
-      </c>
-      <c r="U21" t="s">
-        <v>45</v>
       </c>
       <c r="V21" t="s">
         <v>19</v>
@@ -4468,10 +4468,10 @@
         <v>22</v>
       </c>
       <c r="F22" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="G22" t="s">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="H22" t="s">
         <v>37</v>
@@ -4489,7 +4489,7 @@
         <v>19</v>
       </c>
       <c r="M22" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="N22" t="s">
         <v>143</v>
@@ -4498,22 +4498,22 @@
         <v>100</v>
       </c>
       <c r="P22" t="s">
-        <v>109</v>
+        <v>83</v>
       </c>
       <c r="Q22" t="s">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="R22" t="s">
+        <v>43</v>
+      </c>
+      <c r="S22" t="s">
+        <v>19</v>
+      </c>
+      <c r="T22" t="s">
+        <v>19</v>
+      </c>
+      <c r="U22" t="s">
         <v>44</v>
-      </c>
-      <c r="S22" t="s">
-        <v>19</v>
-      </c>
-      <c r="T22" t="s">
-        <v>19</v>
-      </c>
-      <c r="U22" t="s">
-        <v>45</v>
       </c>
       <c r="V22" t="s">
         <v>19</v>
@@ -4542,16 +4542,16 @@
         <v>22</v>
       </c>
       <c r="F23" t="s">
-        <v>35</v>
+        <v>101</v>
       </c>
       <c r="G23" t="s">
-        <v>46</v>
+        <v>112</v>
       </c>
       <c r="H23" t="s">
         <v>37</v>
       </c>
       <c r="I23" t="s">
-        <v>43</v>
+        <v>106</v>
       </c>
       <c r="J23">
         <v>4</v>
@@ -4563,7 +4563,7 @@
         <v>19</v>
       </c>
       <c r="M23" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="N23" t="s">
         <v>156</v>
@@ -4572,22 +4572,22 @@
         <v>65</v>
       </c>
       <c r="P23" t="s">
-        <v>41</v>
+        <v>104</v>
       </c>
       <c r="Q23" t="s">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="R23" t="s">
+        <v>43</v>
+      </c>
+      <c r="S23" t="s">
+        <v>19</v>
+      </c>
+      <c r="T23" t="s">
+        <v>19</v>
+      </c>
+      <c r="U23" t="s">
         <v>44</v>
-      </c>
-      <c r="S23" t="s">
-        <v>19</v>
-      </c>
-      <c r="T23" t="s">
-        <v>19</v>
-      </c>
-      <c r="U23" t="s">
-        <v>45</v>
       </c>
       <c r="V23" t="s">
         <v>19</v>
@@ -4616,16 +4616,16 @@
         <v>22</v>
       </c>
       <c r="F24" t="s">
-        <v>35</v>
+        <v>101</v>
       </c>
       <c r="G24" t="s">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="H24" t="s">
         <v>37</v>
       </c>
       <c r="I24" t="s">
-        <v>43</v>
+        <v>106</v>
       </c>
       <c r="J24">
         <v>4</v>
@@ -4637,7 +4637,7 @@
         <v>19</v>
       </c>
       <c r="M24" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="N24" t="s">
         <v>140</v>
@@ -4646,22 +4646,22 @@
         <v>100</v>
       </c>
       <c r="P24" t="s">
-        <v>41</v>
+        <v>104</v>
       </c>
       <c r="Q24" t="s">
-        <v>52</v>
+        <v>115</v>
       </c>
       <c r="R24" t="s">
+        <v>43</v>
+      </c>
+      <c r="S24" t="s">
+        <v>19</v>
+      </c>
+      <c r="T24" t="s">
+        <v>19</v>
+      </c>
+      <c r="U24" t="s">
         <v>44</v>
-      </c>
-      <c r="S24" t="s">
-        <v>19</v>
-      </c>
-      <c r="T24" t="s">
-        <v>19</v>
-      </c>
-      <c r="U24" t="s">
-        <v>45</v>
       </c>
       <c r="V24" t="s">
         <v>19</v>
@@ -4684,16 +4684,16 @@
         <v>137</v>
       </c>
       <c r="D25" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="E25" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="F25" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="G25" t="s">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="H25" t="s">
         <v>37</v>
@@ -4711,7 +4711,7 @@
         <v>19</v>
       </c>
       <c r="M25" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="N25" t="s">
         <v>158</v>
@@ -4720,25 +4720,25 @@
         <v>150</v>
       </c>
       <c r="P25" t="s">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="Q25" t="s">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="R25" t="s">
+        <v>43</v>
+      </c>
+      <c r="S25" t="s">
+        <v>19</v>
+      </c>
+      <c r="T25" t="s">
+        <v>19</v>
+      </c>
+      <c r="U25" t="s">
         <v>44</v>
       </c>
-      <c r="S25" t="s">
-        <v>19</v>
-      </c>
-      <c r="T25" t="s">
-        <v>19</v>
-      </c>
-      <c r="U25" t="s">
-        <v>45</v>
-      </c>
       <c r="V25" t="s">
-        <v>84</v>
+        <v>51</v>
       </c>
       <c r="W25" t="s">
         <v>19</v>
@@ -4758,22 +4758,22 @@
         <v>137</v>
       </c>
       <c r="D26" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="E26" t="s">
-        <v>56</v>
+        <v>86</v>
       </c>
       <c r="F26" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="G26" t="s">
-        <v>79</v>
+        <v>36</v>
       </c>
       <c r="H26" t="s">
         <v>37</v>
       </c>
       <c r="I26" t="s">
-        <v>113</v>
+        <v>85</v>
       </c>
       <c r="J26">
         <v>2</v>
@@ -4785,7 +4785,7 @@
         <v>19</v>
       </c>
       <c r="M26" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="N26" t="s">
         <v>158</v>
@@ -4794,13 +4794,13 @@
         <v>150</v>
       </c>
       <c r="P26" t="s">
-        <v>109</v>
+        <v>83</v>
       </c>
       <c r="Q26" t="s">
-        <v>112</v>
+        <v>84</v>
       </c>
       <c r="R26" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S26" t="s">
         <v>19</v>
@@ -4809,10 +4809,10 @@
         <v>19</v>
       </c>
       <c r="U26" t="s">
-        <v>115</v>
+        <v>88</v>
       </c>
       <c r="V26" t="s">
-        <v>116</v>
+        <v>89</v>
       </c>
       <c r="W26" t="s">
         <v>19</v>
@@ -4853,10 +4853,10 @@
         <v>155</v>
       </c>
       <c r="B2" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="C2" t="s">
-        <v>65</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -5151,7 +5151,7 @@
         <v>193</v>
       </c>
       <c r="N3" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="O3" t="s">
         <v>19</v>
@@ -5213,7 +5213,7 @@
         <v>193</v>
       </c>
       <c r="N4" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="O4" t="s">
         <v>19</v>
@@ -5336,7 +5336,7 @@
         <v>203</v>
       </c>
       <c r="B5" t="s">
-        <v>115</v>
+        <v>88</v>
       </c>
       <c r="C5" t="s">
         <v>19</v>
@@ -5396,7 +5396,7 @@
         <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="C8" t="s">
         <v>207</v>
@@ -5436,7 +5436,7 @@
         <v>0</v>
       </c>
       <c r="B10" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="C10" t="s">
         <v>209</v>
@@ -5476,7 +5476,7 @@
         <v>210</v>
       </c>
       <c r="B12" t="s">
-        <v>56</v>
+        <v>86</v>
       </c>
       <c r="C12" t="s">
         <v>212</v>
@@ -5496,7 +5496,7 @@
         <v>210</v>
       </c>
       <c r="B13" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="C13" t="s">
         <v>213</v>
@@ -5536,7 +5536,7 @@
         <v>210</v>
       </c>
       <c r="B15" t="s">
-        <v>85</v>
+        <v>52</v>
       </c>
       <c r="C15" t="s">
         <v>215</v>
@@ -5602,7 +5602,7 @@
         <v>220</v>
       </c>
       <c r="D18" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E18">
         <v>1</v>

</xml_diff>